<commit_message>
Release CADR v4 reproducibility package
</commit_message>
<xml_diff>
--- a/results/benchmark/summary.xlsx
+++ b/results/benchmark/summary.xlsx
@@ -472,7 +472,7 @@
     <col width="20" customWidth="1" min="37" max="37"/>
     <col width="27" customWidth="1" min="38" max="38"/>
     <col width="33" customWidth="1" min="39" max="39"/>
-    <col width="19" customWidth="1" min="40" max="40"/>
+    <col width="15" customWidth="1" min="40" max="40"/>
     <col width="19" customWidth="1" min="41" max="41"/>
     <col width="30" customWidth="1" min="42" max="42"/>
     <col width="25" customWidth="1" min="43" max="43"/>
@@ -750,37 +750,37 @@
         <v>12.82333870967742</v>
       </c>
       <c r="F2" t="n">
-        <v>9.465464516129032</v>
+        <v>9.437125806451613</v>
       </c>
       <c r="G2" t="n">
-        <v>26.18564688628472</v>
+        <v>26.40664011058466</v>
       </c>
       <c r="H2" t="n">
         <v>6.642930107526882</v>
       </c>
       <c r="I2" t="n">
-        <v>4.968096530577958</v>
+        <v>4.940028881048387</v>
       </c>
       <c r="J2" t="n">
-        <v>25.21227154040394</v>
+        <v>25.63479065584319</v>
       </c>
       <c r="K2" t="n">
         <v>1.966609786189553</v>
       </c>
       <c r="L2" t="n">
-        <v>1.929051139169614</v>
+        <v>1.935340600083363</v>
       </c>
       <c r="M2" t="n">
-        <v>1.909816949132093</v>
+        <v>1.590004602121686</v>
       </c>
       <c r="N2" t="n">
-        <v>1246.07618125</v>
+        <v>1266.9585125</v>
       </c>
       <c r="O2" t="n">
         <v>744</v>
       </c>
       <c r="P2" t="n">
-        <v>2199</v>
+        <v>2232</v>
       </c>
       <c r="Q2" t="n">
         <v>0</v>
@@ -804,25 +804,25 @@
         <v>100</v>
       </c>
       <c r="X2" t="n">
-        <v>349.3018</v>
+        <v>361.6945375</v>
       </c>
       <c r="Y2" t="n">
-        <v>1751.62950696992</v>
+        <v>1843.719535799389</v>
       </c>
       <c r="Z2" t="n">
-        <v>4027.978448888944</v>
+        <v>4129.328014649991</v>
       </c>
       <c r="AA2" t="n">
-        <v>2276.348941919024</v>
+        <v>2285.608478850602</v>
       </c>
       <c r="AB2" t="n">
-        <v>2276.348941919025</v>
+        <v>2285.608478850602</v>
       </c>
       <c r="AC2" t="n">
-        <v>1531.618778375492</v>
+        <v>1613.693563873243</v>
       </c>
       <c r="AD2" t="n">
-        <v>1903.983860147258</v>
+        <v>1949.651021361922</v>
       </c>
       <c r="AE2" t="n">
         <v>341</v>
@@ -840,34 +840,34 @@
         <v>22.04301075268817</v>
       </c>
       <c r="AJ2" t="n">
-        <v>288.06315625</v>
+        <v>284.11648125</v>
       </c>
       <c r="AK2" t="n">
-        <v>8.231175</v>
+        <v>8.153524999999998</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.073754023857527</v>
+        <v>1.091212331989247</v>
       </c>
       <c r="AM2" t="n">
         <v>1023.3295</v>
       </c>
       <c r="AN2" t="n">
-        <v>735.26634375</v>
+        <v>739.2130187499999</v>
       </c>
       <c r="AO2" t="n">
-        <v>510.8098375</v>
+        <v>527.7454937499999</v>
       </c>
       <c r="AP2" t="n">
-        <v>288.06315625</v>
+        <v>284.11648125</v>
       </c>
       <c r="AQ2" t="n">
-        <v>59.00653225009231</v>
+        <v>58.34547946572953</v>
       </c>
       <c r="AR2" t="n">
-        <v>71.96786157571857</v>
+        <v>71.45174574135866</v>
       </c>
       <c r="AS2" t="n">
-        <v>2.382306115136825</v>
+        <v>2.494165401628202</v>
       </c>
       <c r="AT2" t="inlineStr">
         <is>
@@ -878,10 +878,10 @@
         <v>19.07025</v>
       </c>
       <c r="AV2" t="n">
-        <v>15.231175</v>
+        <v>15.153525</v>
       </c>
       <c r="AW2" t="n">
-        <v>20.1312253378954</v>
+        <v>20.53840405867778</v>
       </c>
     </row>
     <row r="3">
@@ -912,28 +912,28 @@
         <v>6.642930107526882</v>
       </c>
       <c r="I3" t="n">
-        <v>4.927639919354839</v>
+        <v>4.921923445900537</v>
       </c>
       <c r="J3" t="n">
-        <v>25.82128910597005</v>
+        <v>25.90734259986161</v>
       </c>
       <c r="K3" t="n">
         <v>1.966609786189553</v>
       </c>
       <c r="L3" t="n">
-        <v>1.941058946169134</v>
+        <v>1.94290394431517</v>
       </c>
       <c r="M3" t="n">
-        <v>1.299232832046734</v>
+        <v>1.205416653616614</v>
       </c>
       <c r="N3" t="n">
-        <v>1276.1759</v>
+        <v>1280.42895625</v>
       </c>
       <c r="O3" t="n">
         <v>744</v>
       </c>
       <c r="P3" t="n">
-        <v>2228</v>
+        <v>2230</v>
       </c>
       <c r="Q3" t="n">
         <v>0</v>
@@ -957,70 +957,70 @@
         <v>100</v>
       </c>
       <c r="X3" t="n">
-        <v>371.4990937499999</v>
+        <v>373.4997625</v>
       </c>
       <c r="Y3" t="n">
-        <v>1885.399571309875</v>
+        <v>1876.226235997601</v>
       </c>
       <c r="Z3" t="n">
-        <v>4032.562485560033</v>
+        <v>4217.909634249095</v>
       </c>
       <c r="AA3" t="n">
-        <v>2147.162914250157</v>
+        <v>2341.683398251494</v>
       </c>
       <c r="AB3" t="n">
-        <v>2147.162914250157</v>
+        <v>2341.683398251495</v>
       </c>
       <c r="AC3" t="n">
-        <v>1650.874082962516</v>
+        <v>1642.458876610775</v>
       </c>
       <c r="AD3" t="n">
-        <v>1899.018498606337</v>
+        <v>1992.071137431135</v>
       </c>
       <c r="AE3" t="n">
         <v>341</v>
       </c>
       <c r="AF3" t="n">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AG3" t="n">
         <v>45.83333333333333</v>
       </c>
       <c r="AH3" t="n">
-        <v>23.79032258064516</v>
+        <v>23.65591397849462</v>
       </c>
       <c r="AI3" t="n">
-        <v>22.04301075268817</v>
+        <v>22.17741935483871</v>
       </c>
       <c r="AJ3" t="n">
-        <v>283.93235625</v>
+        <v>283.9348562500001</v>
       </c>
       <c r="AK3" t="n">
         <v>8.153524999999998</v>
       </c>
       <c r="AL3" t="n">
-        <v>1.103106334005376</v>
+        <v>1.108829527889785</v>
       </c>
       <c r="AM3" t="n">
         <v>1023.3295</v>
       </c>
       <c r="AN3" t="n">
-        <v>739.3971437499999</v>
+        <v>739.39464375</v>
       </c>
       <c r="AO3" t="n">
-        <v>536.77875625</v>
+        <v>541.0343124999999</v>
       </c>
       <c r="AP3" t="n">
-        <v>283.93235625</v>
+        <v>283.93485625</v>
       </c>
       <c r="AQ3" t="n">
-        <v>57.9384976436242</v>
+        <v>57.74585463261231</v>
       </c>
       <c r="AR3" t="n">
-        <v>70.88966389742981</v>
+        <v>70.83010652977802</v>
       </c>
       <c r="AS3" t="n">
-        <v>2.549914599003853</v>
+        <v>2.537516672398265</v>
       </c>
       <c r="AT3" t="inlineStr">
         <is>
@@ -1065,28 +1065,28 @@
         <v>6.642930107526882</v>
       </c>
       <c r="I4" t="n">
-        <v>4.928889910954301</v>
+        <v>4.921403461021505</v>
       </c>
       <c r="J4" t="n">
-        <v>25.80247223481186</v>
+        <v>25.91517024324511</v>
       </c>
       <c r="K4" t="n">
         <v>1.966609786189553</v>
       </c>
       <c r="L4" t="n">
-        <v>1.940083162158907</v>
+        <v>1.943067315223592</v>
       </c>
       <c r="M4" t="n">
-        <v>1.348850403213068</v>
+        <v>1.197109418008952</v>
       </c>
       <c r="N4" t="n">
-        <v>1275.24590625</v>
+        <v>1280.815825</v>
       </c>
       <c r="O4" t="n">
         <v>744</v>
       </c>
       <c r="P4" t="n">
-        <v>2228</v>
+        <v>2232</v>
       </c>
       <c r="Q4" t="n">
         <v>0</v>
@@ -1110,25 +1110,25 @@
         <v>100</v>
       </c>
       <c r="X4" t="n">
-        <v>368.53050625</v>
+        <v>373.642175</v>
       </c>
       <c r="Y4" t="n">
-        <v>1879.285908242032</v>
+        <v>1876.33190745596</v>
       </c>
       <c r="Z4" t="n">
-        <v>4129.380818994313</v>
+        <v>4220.92490890847</v>
       </c>
       <c r="AA4" t="n">
-        <v>2250.094910752281</v>
+        <v>2344.59300145251</v>
       </c>
       <c r="AB4" t="n">
-        <v>2250.094910752281</v>
+        <v>2344.59300145251</v>
       </c>
       <c r="AC4" t="n">
-        <v>1645.312346097025</v>
+        <v>1642.545155395186</v>
       </c>
       <c r="AD4" t="n">
-        <v>1947.703628424653</v>
+        <v>1993.569078423848</v>
       </c>
       <c r="AE4" t="n">
         <v>341</v>
@@ -1152,7 +1152,7 @@
         <v>8.153524999999998</v>
       </c>
       <c r="AL4" t="n">
-        <v>1.101205922379032</v>
+        <v>1.108692372311828</v>
       </c>
       <c r="AM4" t="n">
         <v>1023.3295</v>
@@ -1161,19 +1161,19 @@
         <v>739.6391</v>
       </c>
       <c r="AO4" t="n">
-        <v>535.60680625</v>
+        <v>541.176725</v>
       </c>
       <c r="AP4" t="n">
         <v>283.6904</v>
       </c>
       <c r="AQ4" t="n">
-        <v>57.99972353371356</v>
+        <v>57.7474985523387</v>
       </c>
       <c r="AR4" t="n">
-        <v>71.10122020828875</v>
+        <v>70.82779836827828</v>
       </c>
       <c r="AS4" t="n">
-        <v>2.540814713881448</v>
+        <v>2.536820873120364</v>
       </c>
       <c r="AT4" t="inlineStr">
         <is>
@@ -1209,37 +1209,37 @@
         <v>12.0433064516129</v>
       </c>
       <c r="F5" t="n">
-        <v>9.157001411290322</v>
+        <v>9.119811290322581</v>
       </c>
       <c r="G5" t="n">
-        <v>23.96605161480412</v>
+        <v>24.27485485847447</v>
       </c>
       <c r="H5" t="n">
         <v>6.484645833333333</v>
       </c>
       <c r="I5" t="n">
-        <v>4.857953427419355</v>
+        <v>4.828733467741936</v>
       </c>
       <c r="J5" t="n">
-        <v>25.08529297856505</v>
+        <v>25.53589522313513</v>
       </c>
       <c r="K5" t="n">
         <v>1.888227790632866</v>
       </c>
       <c r="L5" t="n">
-        <v>1.903677557400715</v>
+        <v>1.908174481748671</v>
       </c>
       <c r="M5" t="n">
-        <v>-0.8182151986371745</v>
+        <v>-1.056371017032824</v>
       </c>
       <c r="N5" t="n">
-        <v>1210.25915</v>
+        <v>1231.9988</v>
       </c>
       <c r="O5" t="n">
         <v>744</v>
       </c>
       <c r="P5" t="n">
-        <v>2193</v>
+        <v>2232</v>
       </c>
       <c r="Q5" t="n">
         <v>0</v>
@@ -1251,7 +1251,7 @@
         <v>2</v>
       </c>
       <c r="T5" t="n">
-        <v>0.09119927040583675</v>
+        <v>0.08960573476702509</v>
       </c>
       <c r="U5" t="n">
         <v>409</v>
@@ -1263,70 +1263,70 @@
         <v>100</v>
       </c>
       <c r="X5" t="n">
-        <v>395.52620625</v>
+        <v>408.65355</v>
       </c>
       <c r="Y5" t="n">
-        <v>2070.310236121836</v>
+        <v>2201.616662105195</v>
       </c>
       <c r="Z5" t="n">
-        <v>3174.495563967187</v>
+        <v>3252.221128535937</v>
       </c>
       <c r="AA5" t="n">
-        <v>1104.185327845351</v>
+        <v>1050.604466430742</v>
       </c>
       <c r="AB5" t="n">
-        <v>1104.185327845351</v>
+        <v>1050.604466430742</v>
       </c>
       <c r="AC5" t="n">
-        <v>1821.083516713761</v>
+        <v>1938.375406145216</v>
       </c>
       <c r="AD5" t="n">
-        <v>1462.634422279556</v>
+        <v>1494.489936287979</v>
       </c>
       <c r="AE5" t="n">
         <v>335</v>
       </c>
       <c r="AF5" t="n">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="AG5" t="n">
         <v>45.0268817204301</v>
       </c>
       <c r="AH5" t="n">
-        <v>16.8010752688172</v>
+        <v>16.26344086021505</v>
       </c>
       <c r="AI5" t="n">
-        <v>28.22580645161291</v>
+        <v>28.76344086021506</v>
       </c>
       <c r="AJ5" t="n">
-        <v>191.48985625</v>
+        <v>186.8098875</v>
       </c>
       <c r="AK5" t="n">
-        <v>6.685587499999999</v>
+        <v>6.602374999999999</v>
       </c>
       <c r="AL5" t="n">
-        <v>1.069427234543011</v>
+        <v>1.086066633064516</v>
       </c>
       <c r="AM5" t="n">
         <v>797.585</v>
       </c>
       <c r="AN5" t="n">
-        <v>606.09514375</v>
+        <v>610.7751125</v>
       </c>
       <c r="AO5" t="n">
-        <v>604.1640062500001</v>
+        <v>621.2236875</v>
       </c>
       <c r="AP5" t="n">
-        <v>191.48985625</v>
+        <v>186.8098875</v>
       </c>
       <c r="AQ5" t="n">
-        <v>50.0797819830571</v>
+        <v>49.57595027689963</v>
       </c>
       <c r="AR5" t="n">
-        <v>67.31888321191374</v>
+        <v>66.83003668510067</v>
       </c>
       <c r="AS5" t="n">
-        <v>3.415817231783976</v>
+        <v>3.6046273285328</v>
       </c>
       <c r="AT5" t="inlineStr">
         <is>
@@ -1337,10 +1337,10 @@
         <v>15.11375</v>
       </c>
       <c r="AV5" t="n">
-        <v>13.6855875</v>
+        <v>13.602375</v>
       </c>
       <c r="AW5" t="n">
-        <v>9.449425192291795</v>
+        <v>10.00000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -1371,28 +1371,28 @@
         <v>6.484645833333333</v>
       </c>
       <c r="I6" t="n">
-        <v>4.811650890456989</v>
+        <v>4.80841047547043</v>
       </c>
       <c r="J6" t="n">
-        <v>25.79932637610784</v>
+        <v>25.84929695383626</v>
       </c>
       <c r="K6" t="n">
         <v>1.888227790632866</v>
       </c>
       <c r="L6" t="n">
-        <v>1.914810166968486</v>
+        <v>1.916340446960001</v>
       </c>
       <c r="M6" t="n">
-        <v>-1.407794995259031</v>
+        <v>-1.488838182903368</v>
       </c>
       <c r="N6" t="n">
-        <v>1244.7082375</v>
+        <v>1247.11910625</v>
       </c>
       <c r="O6" t="n">
         <v>744</v>
       </c>
       <c r="P6" t="n">
-        <v>2229</v>
+        <v>2230</v>
       </c>
       <c r="Q6" t="n">
         <v>0</v>
@@ -1401,10 +1401,10 @@
         <v>0</v>
       </c>
       <c r="S6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T6" t="n">
-        <v>0.04486316733961417</v>
+        <v>0.08968609865470852</v>
       </c>
       <c r="U6" t="n">
         <v>409</v>
@@ -1416,25 +1416,25 @@
         <v>100</v>
       </c>
       <c r="X6" t="n">
-        <v>418.20691875</v>
+        <v>420.17989375</v>
       </c>
       <c r="Y6" t="n">
-        <v>2227.609443021797</v>
+        <v>2243.022792875625</v>
       </c>
       <c r="Z6" t="n">
-        <v>3241.522613398437</v>
+        <v>3323.9645381</v>
       </c>
       <c r="AA6" t="n">
-        <v>1013.913170376641</v>
+        <v>1080.941745224375</v>
       </c>
       <c r="AB6" t="n">
-        <v>1013.913170376641</v>
+        <v>1080.941745224375</v>
       </c>
       <c r="AC6" t="n">
-        <v>1961.213477164934</v>
+        <v>1975.020543951191</v>
       </c>
       <c r="AD6" t="n">
-        <v>1487.563323770788</v>
+        <v>1527.981144587783</v>
       </c>
       <c r="AE6" t="n">
         <v>335</v>
@@ -1452,34 +1452,34 @@
         <v>28.76344086021506</v>
       </c>
       <c r="AJ6" t="n">
-        <v>187.29615625</v>
+        <v>186.8582625</v>
       </c>
       <c r="AK6" t="n">
         <v>6.602374999999999</v>
       </c>
       <c r="AL6" t="n">
-        <v>1.104456384408602</v>
+        <v>1.106519665658602</v>
       </c>
       <c r="AM6" t="n">
         <v>797.585</v>
       </c>
       <c r="AN6" t="n">
-        <v>610.28884375</v>
+        <v>610.7267375</v>
       </c>
       <c r="AO6" t="n">
-        <v>634.4193937499999</v>
+        <v>636.3923687500001</v>
       </c>
       <c r="AP6" t="n">
-        <v>187.29615625</v>
+        <v>186.8582625</v>
       </c>
       <c r="AQ6" t="n">
-        <v>49.03067444751284</v>
+        <v>48.97100320565312</v>
       </c>
       <c r="AR6" t="n">
-        <v>66.40120904237206</v>
+        <v>66.3079579452959</v>
       </c>
       <c r="AS6" t="n">
-        <v>3.65009038889513</v>
+        <v>3.672710977183351</v>
       </c>
       <c r="AT6" t="inlineStr">
         <is>
@@ -1524,28 +1524,28 @@
         <v>6.484645833333333</v>
       </c>
       <c r="I7" t="n">
-        <v>4.815625739247312</v>
+        <v>4.808297757056452</v>
       </c>
       <c r="J7" t="n">
-        <v>25.73803006336411</v>
+        <v>25.85103518930626</v>
       </c>
       <c r="K7" t="n">
         <v>1.888227790632866</v>
       </c>
       <c r="L7" t="n">
-        <v>1.913178329483012</v>
+        <v>1.916369039545121</v>
       </c>
       <c r="M7" t="n">
-        <v>-1.321373351982237</v>
+        <v>-1.490352437976927</v>
       </c>
       <c r="N7" t="n">
-        <v>1241.75095</v>
+        <v>1247.20296875</v>
       </c>
       <c r="O7" t="n">
         <v>744</v>
       </c>
       <c r="P7" t="n">
-        <v>2230</v>
+        <v>2232</v>
       </c>
       <c r="Q7" t="n">
         <v>0</v>
@@ -1557,7 +1557,7 @@
         <v>2</v>
       </c>
       <c r="T7" t="n">
-        <v>0.08968609865470852</v>
+        <v>0.08960573476702509</v>
       </c>
       <c r="U7" t="n">
         <v>409</v>
@@ -1569,25 +1569,25 @@
         <v>100</v>
       </c>
       <c r="X7" t="n">
-        <v>414.8988625</v>
+        <v>420.17356875</v>
       </c>
       <c r="Y7" t="n">
-        <v>2221.265868599063</v>
+        <v>2243.196594818203</v>
       </c>
       <c r="Z7" t="n">
-        <v>3249.62189971875</v>
+        <v>3324.241818851562</v>
       </c>
       <c r="AA7" t="n">
-        <v>1028.356031119687</v>
+        <v>1081.045224033359</v>
       </c>
       <c r="AB7" t="n">
-        <v>1028.356031119687</v>
+        <v>1081.045224033359</v>
       </c>
       <c r="AC7" t="n">
-        <v>1955.550799826846</v>
+        <v>1975.176077320619</v>
       </c>
       <c r="AD7" t="n">
-        <v>1491.953415473267</v>
+        <v>1528.110650676989</v>
       </c>
       <c r="AE7" t="n">
         <v>335</v>
@@ -1605,34 +1605,34 @@
         <v>28.76344086021506</v>
       </c>
       <c r="AJ7" t="n">
-        <v>186.9453875</v>
+        <v>186.768075</v>
       </c>
       <c r="AK7" t="n">
         <v>6.602374999999999</v>
       </c>
       <c r="AL7" t="n">
-        <v>1.099538608870968</v>
+        <v>1.106389944556452</v>
       </c>
       <c r="AM7" t="n">
         <v>797.585</v>
       </c>
       <c r="AN7" t="n">
-        <v>610.6396124999999</v>
+        <v>610.816925</v>
       </c>
       <c r="AO7" t="n">
-        <v>631.1113375</v>
+        <v>636.38604375</v>
       </c>
       <c r="AP7" t="n">
-        <v>186.9453875</v>
+        <v>186.768075</v>
       </c>
       <c r="AQ7" t="n">
-        <v>49.17569118831759</v>
+        <v>48.97494155359387</v>
       </c>
       <c r="AR7" t="n">
-        <v>66.58759451724197</v>
+        <v>66.31073054844346</v>
       </c>
       <c r="AS7" t="n">
-        <v>3.637605263610479</v>
+        <v>3.672453239271658</v>
       </c>
       <c r="AT7" t="inlineStr">
         <is>
@@ -1668,37 +1668,37 @@
         <v>5.087908333333332</v>
       </c>
       <c r="F8" t="n">
-        <v>3.681453125</v>
+        <v>3.665249166666667</v>
       </c>
       <c r="G8" t="n">
-        <v>27.64309252820001</v>
+        <v>27.96157228985714</v>
       </c>
       <c r="H8" t="n">
         <v>1.71905</v>
       </c>
       <c r="I8" t="n">
-        <v>1.266953602430556</v>
+        <v>1.257770920138889</v>
       </c>
       <c r="J8" t="n">
-        <v>26.29919999822252</v>
+        <v>26.8333719124581</v>
       </c>
       <c r="K8" t="n">
         <v>3.021445296483412</v>
       </c>
       <c r="L8" t="n">
-        <v>2.950840950955322</v>
+        <v>2.969249648454104</v>
       </c>
       <c r="M8" t="n">
-        <v>2.336773914466162</v>
+        <v>1.727505975039728</v>
       </c>
       <c r="N8" t="n">
-        <v>325.50940625</v>
+        <v>332.1209375</v>
       </c>
       <c r="O8" t="n">
         <v>720</v>
       </c>
       <c r="P8" t="n">
-        <v>2057</v>
+        <v>2160</v>
       </c>
       <c r="Q8" t="n">
         <v>1</v>
@@ -1707,10 +1707,10 @@
         <v>0.1388888888888889</v>
       </c>
       <c r="S8" t="n">
-        <v>317</v>
+        <v>337</v>
       </c>
       <c r="T8" t="n">
-        <v>15.41079241614001</v>
+        <v>15.60185185185185</v>
       </c>
       <c r="U8" t="n">
         <v>716</v>
@@ -1722,25 +1722,25 @@
         <v>100</v>
       </c>
       <c r="X8" t="n">
-        <v>314.42748125</v>
+        <v>321.0390125</v>
       </c>
       <c r="Y8" t="n">
-        <v>458.6090682438653</v>
+        <v>488.8222426560772</v>
       </c>
       <c r="Z8" t="n">
-        <v>967.9858473513925</v>
+        <v>1006.887396834205</v>
       </c>
       <c r="AA8" t="n">
-        <v>509.3767791075272</v>
+        <v>518.0651541781278</v>
       </c>
       <c r="AB8" t="n">
-        <v>509.3767791075272</v>
+        <v>518.0651541781278</v>
       </c>
       <c r="AC8" t="n">
-        <v>404.8383385241723</v>
+        <v>431.9380191112659</v>
       </c>
       <c r="AD8" t="n">
-        <v>457.1075588158497</v>
+        <v>475.0015866446969</v>
       </c>
       <c r="AE8" t="n">
         <v>4</v>
@@ -1764,7 +1764,7 @@
         <v>0.6039249999999994</v>
       </c>
       <c r="AL8" t="n">
-        <v>0.4413576475694444</v>
+        <v>0.4505403298611111</v>
       </c>
       <c r="AM8" t="n">
         <v>8.93975</v>
@@ -1773,19 +1773,19 @@
         <v>8.335825</v>
       </c>
       <c r="AO8" t="n">
-        <v>317.17358125</v>
+        <v>323.7851125</v>
       </c>
       <c r="AP8" t="n">
         <v>0.6039250000000003</v>
       </c>
       <c r="AQ8" t="n">
-        <v>2.560855336265724</v>
+        <v>2.509876391036022</v>
       </c>
       <c r="AR8" t="n">
-        <v>3.404486871107124</v>
+        <v>3.33671375355551</v>
       </c>
       <c r="AS8" t="n">
-        <v>55.01663821443772</v>
+        <v>58.64113541923891</v>
       </c>
       <c r="AT8" t="inlineStr">
         <is>
@@ -1821,37 +1821,37 @@
         <v>5.087908333333332</v>
       </c>
       <c r="F9" t="n">
-        <v>3.681603333333334</v>
+        <v>3.661854583333334</v>
       </c>
       <c r="G9" t="n">
-        <v>27.64014026720212</v>
+        <v>28.02829093160415</v>
       </c>
       <c r="H9" t="n">
         <v>1.71905</v>
       </c>
       <c r="I9" t="n">
-        <v>1.271004340277778</v>
+        <v>1.250525859375</v>
       </c>
       <c r="J9" t="n">
-        <v>26.06356183486355</v>
+        <v>27.25482915709258</v>
       </c>
       <c r="K9" t="n">
         <v>3.021445296483412</v>
       </c>
       <c r="L9" t="n">
-        <v>2.941156145692285</v>
+        <v>2.982710381415455</v>
       </c>
       <c r="M9" t="n">
-        <v>2.657309430178099</v>
+        <v>1.281999548793387</v>
       </c>
       <c r="N9" t="n">
-        <v>322.592875</v>
+        <v>337.33738125</v>
       </c>
       <c r="O9" t="n">
         <v>720</v>
       </c>
       <c r="P9" t="n">
-        <v>2062</v>
+        <v>2159</v>
       </c>
       <c r="Q9" t="n">
         <v>1</v>
@@ -1860,10 +1860,10 @@
         <v>0.1388888888888889</v>
       </c>
       <c r="S9" t="n">
-        <v>285</v>
+        <v>337</v>
       </c>
       <c r="T9" t="n">
-        <v>13.82153249272551</v>
+        <v>15.60907827698009</v>
       </c>
       <c r="U9" t="n">
         <v>716</v>
@@ -1875,25 +1875,25 @@
         <v>100</v>
       </c>
       <c r="X9" t="n">
-        <v>311.51095</v>
+        <v>326.25545625</v>
       </c>
       <c r="Y9" t="n">
-        <v>461.2973873188162</v>
+        <v>500.5611101230199</v>
       </c>
       <c r="Z9" t="n">
-        <v>978.1347213801125</v>
+        <v>1027.83688804983</v>
       </c>
       <c r="AA9" t="n">
-        <v>516.8373340612964</v>
+        <v>527.2757779268102</v>
       </c>
       <c r="AB9" t="n">
-        <v>516.8373340612964</v>
+        <v>527.27577792681</v>
       </c>
       <c r="AC9" t="n">
-        <v>407.3739200391661</v>
+        <v>442.3788308993466</v>
       </c>
       <c r="AD9" t="n">
-        <v>462.1056270502312</v>
+        <v>484.8273044130783</v>
       </c>
       <c r="AE9" t="n">
         <v>4</v>
@@ -1917,7 +1917,7 @@
         <v>0.6039249999999994</v>
       </c>
       <c r="AL9" t="n">
-        <v>0.4373069097222222</v>
+        <v>0.457785390625</v>
       </c>
       <c r="AM9" t="n">
         <v>8.93975</v>
@@ -1926,19 +1926,19 @@
         <v>8.335825</v>
       </c>
       <c r="AO9" t="n">
-        <v>314.25705</v>
+        <v>329.00155625</v>
       </c>
       <c r="AP9" t="n">
         <v>0.6039250000000003</v>
       </c>
       <c r="AQ9" t="n">
-        <v>2.584007783804897</v>
+        <v>2.471064715422788</v>
       </c>
       <c r="AR9" t="n">
-        <v>3.435266510458422</v>
+        <v>3.285116211828066</v>
       </c>
       <c r="AS9" t="n">
-        <v>55.3391400753754</v>
+        <v>60.04937845060567</v>
       </c>
       <c r="AT9" t="inlineStr">
         <is>
@@ -1974,37 +1974,37 @@
         <v>5.087908333333332</v>
       </c>
       <c r="F10" t="n">
-        <v>3.667258750000001</v>
+        <v>3.660469166666667</v>
       </c>
       <c r="G10" t="n">
-        <v>27.92207505048732</v>
+        <v>28.05552052333226</v>
       </c>
       <c r="H10" t="n">
         <v>1.71905</v>
       </c>
       <c r="I10" t="n">
-        <v>1.267180928819444</v>
+        <v>1.250416657986111</v>
       </c>
       <c r="J10" t="n">
-        <v>26.2859760437774</v>
+        <v>27.26118158365893</v>
       </c>
       <c r="K10" t="n">
         <v>3.021445296483412</v>
       </c>
       <c r="L10" t="n">
-        <v>2.930153742566731</v>
+        <v>2.981857642330396</v>
       </c>
       <c r="M10" t="n">
-        <v>3.021453144391929</v>
+        <v>1.310222435570517</v>
       </c>
       <c r="N10" t="n">
-        <v>325.34573125</v>
+        <v>337.41600625</v>
       </c>
       <c r="O10" t="n">
         <v>720</v>
       </c>
       <c r="P10" t="n">
-        <v>2127</v>
+        <v>2160</v>
       </c>
       <c r="Q10" t="n">
         <v>1</v>
@@ -2013,10 +2013,10 @@
         <v>0.1388888888888889</v>
       </c>
       <c r="S10" t="n">
-        <v>327</v>
+        <v>337</v>
       </c>
       <c r="T10" t="n">
-        <v>15.3737658674189</v>
+        <v>15.60185185185185</v>
       </c>
       <c r="U10" t="n">
         <v>716</v>
@@ -2028,25 +2028,25 @@
         <v>100</v>
       </c>
       <c r="X10" t="n">
-        <v>314.26380625</v>
+        <v>326.33408125</v>
       </c>
       <c r="Y10" t="n">
-        <v>460.9186732987057</v>
+        <v>500.7786435973168</v>
       </c>
       <c r="Z10" t="n">
-        <v>976.5469300156888</v>
+        <v>1028.216367184205</v>
       </c>
       <c r="AA10" t="n">
-        <v>515.6282567169831</v>
+        <v>527.4377235868881</v>
       </c>
       <c r="AB10" t="n">
-        <v>515.6282567169829</v>
+        <v>527.4377235868881</v>
       </c>
       <c r="AC10" t="n">
-        <v>406.9012560527246</v>
+        <v>442.5734985211225</v>
       </c>
       <c r="AD10" t="n">
-        <v>461.2647563848539</v>
+        <v>485.0056110540053</v>
       </c>
       <c r="AE10" t="n">
         <v>4</v>
@@ -2070,7 +2070,7 @@
         <v>0.6039249999999994</v>
       </c>
       <c r="AL10" t="n">
-        <v>0.4411303211805555</v>
+        <v>0.4578945920138889</v>
       </c>
       <c r="AM10" t="n">
         <v>8.93975</v>
@@ -2079,19 +2079,19 @@
         <v>8.335825</v>
       </c>
       <c r="AO10" t="n">
-        <v>317.00990625</v>
+        <v>329.08018125</v>
       </c>
       <c r="AP10" t="n">
         <v>0.6039250000000003</v>
       </c>
       <c r="AQ10" t="n">
-        <v>2.562143651915519</v>
+        <v>2.470488905562997</v>
       </c>
       <c r="AR10" t="n">
-        <v>3.406199601089741</v>
+        <v>3.284350710911184</v>
       </c>
       <c r="AS10" t="n">
-        <v>55.29370797715951</v>
+        <v>60.07547466475326</v>
       </c>
       <c r="AT10" t="inlineStr">
         <is>
@@ -2262,16 +2262,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>9.446572043010752</v>
+        <v>9.437125806451613</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0163613616607444</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>9.437125806451613</v>
       </c>
       <c r="F5" t="n">
-        <v>9.465464516129032</v>
+        <v>9.437125806451613</v>
       </c>
       <c r="G5" t="n">
         <v>3</v>
@@ -2289,13 +2289,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>26.33297570248468</v>
+        <v>26.40664011058466</v>
       </c>
       <c r="D6" t="n">
-        <v>0.127590497538655</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>26.18564688628472</v>
+        <v>26.40664011058466</v>
       </c>
       <c r="F6" t="n">
         <v>26.40664011058466</v>
@@ -2343,16 +2343,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>4.9415421202957</v>
+        <v>4.927785262656809</v>
       </c>
       <c r="D8" t="n">
-        <v>0.02300528523684436</v>
+        <v>0.01060647158849398</v>
       </c>
       <c r="E8" t="n">
-        <v>4.927639919354839</v>
+        <v>4.921403461021505</v>
       </c>
       <c r="F8" t="n">
-        <v>4.968096530577958</v>
+        <v>4.940028881048387</v>
       </c>
       <c r="G8" t="n">
         <v>3</v>
@@ -2370,16 +2370,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>25.61201096039528</v>
+        <v>25.81910116631664</v>
       </c>
       <c r="D9" t="n">
-        <v>0.3463123179751297</v>
+        <v>0.1596655604802483</v>
       </c>
       <c r="E9" t="n">
-        <v>25.21227154040394</v>
+        <v>25.63479065584319</v>
       </c>
       <c r="F9" t="n">
-        <v>25.82128910597005</v>
+        <v>25.91517024324511</v>
       </c>
       <c r="G9" t="n">
         <v>3</v>
@@ -2424,16 +2424,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1.936731082499218</v>
+        <v>1.940437286540708</v>
       </c>
       <c r="D11" t="n">
-        <v>0.006668896892898054</v>
+        <v>0.004414615741692032</v>
       </c>
       <c r="E11" t="n">
-        <v>1.929051139169614</v>
+        <v>1.935340600083363</v>
       </c>
       <c r="F11" t="n">
-        <v>1.941058946169134</v>
+        <v>1.943067315223592</v>
       </c>
       <c r="G11" t="n">
         <v>3</v>
@@ -2451,16 +2451,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1.519300061463965</v>
+        <v>1.330843557915751</v>
       </c>
       <c r="D12" t="n">
-        <v>0.3391062599062609</v>
+        <v>0.2244784792943265</v>
       </c>
       <c r="E12" t="n">
-        <v>1.299232832046734</v>
+        <v>1.197109418008952</v>
       </c>
       <c r="F12" t="n">
-        <v>1.909816949132093</v>
+        <v>1.590004602121686</v>
       </c>
       <c r="G12" t="n">
         <v>3</v>
@@ -2478,16 +2478,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1265.8326625</v>
+        <v>1276.067764583333</v>
       </c>
       <c r="D13" t="n">
-        <v>17.1159322162119</v>
+        <v>7.891214861839402</v>
       </c>
       <c r="E13" t="n">
-        <v>1246.07618125</v>
+        <v>1266.9585125</v>
       </c>
       <c r="F13" t="n">
-        <v>1276.1759</v>
+        <v>1280.815825</v>
       </c>
       <c r="G13" t="n">
         <v>3</v>
@@ -2532,16 +2532,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2218.333333333333</v>
+        <v>2231.333333333333</v>
       </c>
       <c r="D15" t="n">
-        <v>16.74315780649914</v>
+        <v>1.154700538379252</v>
       </c>
       <c r="E15" t="n">
-        <v>2199</v>
+        <v>2230</v>
       </c>
       <c r="F15" t="n">
-        <v>2228</v>
+        <v>2232</v>
       </c>
       <c r="G15" t="n">
         <v>3</v>
@@ -2748,16 +2748,16 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>363.1104666666666</v>
+        <v>369.6121583333334</v>
       </c>
       <c r="D23" t="n">
-        <v>12.05041842715932</v>
+        <v>6.857230496006703</v>
       </c>
       <c r="E23" t="n">
-        <v>349.3018</v>
+        <v>361.6945375</v>
       </c>
       <c r="F23" t="n">
-        <v>371.4990937499999</v>
+        <v>373.642175</v>
       </c>
       <c r="G23" t="n">
         <v>3</v>
@@ -2775,16 +2775,16 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1838.771662173942</v>
+        <v>1865.425893084316</v>
       </c>
       <c r="D24" t="n">
-        <v>75.52920381698871</v>
+        <v>18.79833108416747</v>
       </c>
       <c r="E24" t="n">
-        <v>1751.62950696992</v>
+        <v>1843.719535799389</v>
       </c>
       <c r="F24" t="n">
-        <v>1885.399571309875</v>
+        <v>1876.33190745596</v>
       </c>
       <c r="G24" t="n">
         <v>3</v>
@@ -2802,16 +2802,16 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>4063.307251147764</v>
+        <v>4189.387519269185</v>
       </c>
       <c r="D25" t="n">
-        <v>57.26727358649015</v>
+        <v>52.03490214889539</v>
       </c>
       <c r="E25" t="n">
-        <v>4027.978448888944</v>
+        <v>4129.328014649991</v>
       </c>
       <c r="F25" t="n">
-        <v>4129.380818994313</v>
+        <v>4220.92490890847</v>
       </c>
       <c r="G25" t="n">
         <v>3</v>
@@ -2829,16 +2829,16 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2224.535588973821</v>
+        <v>2323.961626184869</v>
       </c>
       <c r="D26" t="n">
-        <v>68.28042643061396</v>
+        <v>33.24664465069861</v>
       </c>
       <c r="E26" t="n">
-        <v>2147.162914250157</v>
+        <v>2285.608478850602</v>
       </c>
       <c r="F26" t="n">
-        <v>2276.348941919024</v>
+        <v>2344.59300145251</v>
       </c>
       <c r="G26" t="n">
         <v>3</v>
@@ -2856,16 +2856,16 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2224.535588973821</v>
+        <v>2323.961626184869</v>
       </c>
       <c r="D27" t="n">
-        <v>68.28042643061431</v>
+        <v>33.24664465069885</v>
       </c>
       <c r="E27" t="n">
-        <v>2147.162914250157</v>
+        <v>2285.608478850602</v>
       </c>
       <c r="F27" t="n">
-        <v>2276.348941919025</v>
+        <v>2344.59300145251</v>
       </c>
       <c r="G27" t="n">
         <v>3</v>
@@ -2883,16 +2883,16 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1609.268402478344</v>
+        <v>1632.899198626401</v>
       </c>
       <c r="D28" t="n">
-        <v>67.30402158657346</v>
+        <v>16.63262353662079</v>
       </c>
       <c r="E28" t="n">
-        <v>1531.618778375492</v>
+        <v>1613.693563873243</v>
       </c>
       <c r="F28" t="n">
-        <v>1650.874082962516</v>
+        <v>1642.545155395186</v>
       </c>
       <c r="G28" t="n">
         <v>3</v>
@@ -2910,16 +2910,16 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1916.901995726083</v>
+        <v>1978.430412405635</v>
       </c>
       <c r="D29" t="n">
-        <v>26.79028063461157</v>
+        <v>24.93493469892439</v>
       </c>
       <c r="E29" t="n">
-        <v>1899.018498606337</v>
+        <v>1949.651021361922</v>
       </c>
       <c r="F29" t="n">
-        <v>1947.703628424653</v>
+        <v>1993.569078423848</v>
       </c>
       <c r="G29" t="n">
         <v>3</v>
@@ -2964,7 +2964,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>176.6666666666667</v>
+        <v>176.3333333333333</v>
       </c>
       <c r="D31" t="n">
         <v>0.5773502691896258</v>
@@ -3018,7 +3018,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>23.74551971326165</v>
+        <v>23.70071684587813</v>
       </c>
       <c r="D33" t="n">
         <v>0.07760084263301543</v>
@@ -3045,7 +3045,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>22.08781362007168</v>
+        <v>22.1326164874552</v>
       </c>
       <c r="D34" t="n">
         <v>0.07760084263301747</v>
@@ -3072,16 +3072,16 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>285.2286375</v>
+        <v>283.9139125000001</v>
       </c>
       <c r="D35" t="n">
-        <v>2.457744517805819</v>
+        <v>0.2138113383298706</v>
       </c>
       <c r="E35" t="n">
         <v>283.6904000000001</v>
       </c>
       <c r="F35" t="n">
-        <v>288.06315625</v>
+        <v>284.11648125</v>
       </c>
       <c r="G35" t="n">
         <v>3</v>
@@ -3099,16 +3099,16 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>8.179408333333333</v>
+        <v>8.153524999999998</v>
       </c>
       <c r="D36" t="n">
-        <v>0.0448312484025756</v>
+        <v>0</v>
       </c>
       <c r="E36" t="n">
         <v>8.153524999999998</v>
       </c>
       <c r="F36" t="n">
-        <v>8.231175</v>
+        <v>8.153524999999998</v>
       </c>
       <c r="G36" t="n">
         <v>3</v>
@@ -3126,16 +3126,16 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1.092688760080645</v>
+        <v>1.102911410730287</v>
       </c>
       <c r="D37" t="n">
-        <v>0.01642547009880324</v>
+        <v>0.01013193147701493</v>
       </c>
       <c r="E37" t="n">
-        <v>1.073754023857527</v>
+        <v>1.091212331989247</v>
       </c>
       <c r="F37" t="n">
-        <v>1.103106334005376</v>
+        <v>1.108829527889785</v>
       </c>
       <c r="G37" t="n">
         <v>3</v>
@@ -3180,13 +3180,13 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>738.1008624999999</v>
+        <v>739.4155875</v>
       </c>
       <c r="D39" t="n">
-        <v>2.457744517805806</v>
+        <v>0.2138113383299514</v>
       </c>
       <c r="E39" t="n">
-        <v>735.26634375</v>
+        <v>739.2130187499999</v>
       </c>
       <c r="F39" t="n">
         <v>739.6391</v>
@@ -3207,16 +3207,16 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>527.7318</v>
+        <v>536.6521770833333</v>
       </c>
       <c r="D40" t="n">
-        <v>14.66655985018912</v>
+        <v>7.713742692769054</v>
       </c>
       <c r="E40" t="n">
-        <v>510.8098375</v>
+        <v>527.7454937499999</v>
       </c>
       <c r="F40" t="n">
-        <v>536.77875625</v>
+        <v>541.176725</v>
       </c>
       <c r="G40" t="n">
         <v>3</v>
@@ -3234,16 +3234,16 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>285.2286375</v>
+        <v>283.9139125</v>
       </c>
       <c r="D41" t="n">
-        <v>2.457744517805854</v>
+        <v>0.2138113383299245</v>
       </c>
       <c r="E41" t="n">
         <v>283.6904</v>
       </c>
       <c r="F41" t="n">
-        <v>288.06315625</v>
+        <v>284.11648125</v>
       </c>
       <c r="G41" t="n">
         <v>3</v>
@@ -3261,16 +3261,16 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>58.31491780914336</v>
+        <v>57.94627755022685</v>
       </c>
       <c r="D42" t="n">
-        <v>0.5997374872401745</v>
+        <v>0.3457199771835254</v>
       </c>
       <c r="E42" t="n">
-        <v>57.9384976436242</v>
+        <v>57.74585463261231</v>
       </c>
       <c r="F42" t="n">
-        <v>59.00653225009231</v>
+        <v>58.34547946572953</v>
       </c>
       <c r="G42" t="n">
         <v>3</v>
@@ -3288,16 +3288,16 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>71.31958189381237</v>
+        <v>71.03655021313833</v>
       </c>
       <c r="D43" t="n">
-        <v>0.5713045839526912</v>
+        <v>0.3595717270490047</v>
       </c>
       <c r="E43" t="n">
-        <v>70.88966389742981</v>
+        <v>70.82779836827828</v>
       </c>
       <c r="F43" t="n">
-        <v>71.96786157571857</v>
+        <v>71.45174574135866</v>
       </c>
       <c r="G43" t="n">
         <v>3</v>
@@ -3315,16 +3315,16 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2.491011809340709</v>
+        <v>2.52283431571561</v>
       </c>
       <c r="D44" t="n">
-        <v>0.09425177951408351</v>
+        <v>0.02483044523105024</v>
       </c>
       <c r="E44" t="n">
-        <v>2.382306115136825</v>
+        <v>2.494165401628202</v>
       </c>
       <c r="F44" t="n">
-        <v>2.549914599003853</v>
+        <v>2.537516672398265</v>
       </c>
       <c r="G44" t="n">
         <v>3</v>
@@ -3369,16 +3369,16 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>15.17940833333333</v>
+        <v>15.153525</v>
       </c>
       <c r="D46" t="n">
-        <v>0.04483124840257457</v>
+        <v>0</v>
       </c>
       <c r="E46" t="n">
         <v>15.153525</v>
       </c>
       <c r="F46" t="n">
-        <v>15.231175</v>
+        <v>15.153525</v>
       </c>
       <c r="G46" t="n">
         <v>3</v>
@@ -3396,13 +3396,13 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>20.40267781841699</v>
+        <v>20.53840405867778</v>
       </c>
       <c r="D47" t="n">
-        <v>0.2350847440519943</v>
+        <v>0</v>
       </c>
       <c r="E47" t="n">
-        <v>20.1312253378954</v>
+        <v>20.53840405867778</v>
       </c>
       <c r="F47" t="n">
         <v>20.53840405867778</v>
@@ -3504,16 +3504,16 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>9.132207997311829</v>
+        <v>9.119811290322581</v>
       </c>
       <c r="D51" t="n">
-        <v>0.02147172635192026</v>
+        <v>0</v>
       </c>
       <c r="E51" t="n">
         <v>9.119811290322581</v>
       </c>
       <c r="F51" t="n">
-        <v>9.157001411290322</v>
+        <v>9.119811290322581</v>
       </c>
       <c r="G51" t="n">
         <v>3</v>
@@ -3531,13 +3531,13 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>24.17192044391768</v>
+        <v>24.27485485847447</v>
       </c>
       <c r="D52" t="n">
-        <v>0.1782876358597066</v>
+        <v>0</v>
       </c>
       <c r="E52" t="n">
-        <v>23.96605161480412</v>
+        <v>24.27485485847447</v>
       </c>
       <c r="F52" t="n">
         <v>24.27485485847447</v>
@@ -3585,16 +3585,16 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>4.828410019041219</v>
+        <v>4.815147233422938</v>
       </c>
       <c r="D54" t="n">
-        <v>0.02566241589707575</v>
+        <v>0.01176615904142967</v>
       </c>
       <c r="E54" t="n">
-        <v>4.811650890456989</v>
+        <v>4.808297757056452</v>
       </c>
       <c r="F54" t="n">
-        <v>4.857953427419355</v>
+        <v>4.828733467741936</v>
       </c>
       <c r="G54" t="n">
         <v>3</v>
@@ -3612,16 +3612,16 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>25.54088313934567</v>
+        <v>25.74540912209255</v>
       </c>
       <c r="D55" t="n">
-        <v>0.3957412101854886</v>
+        <v>0.1814464404663031</v>
       </c>
       <c r="E55" t="n">
-        <v>25.08529297856505</v>
+        <v>25.53589522313513</v>
       </c>
       <c r="F55" t="n">
-        <v>25.79932637610784</v>
+        <v>25.85103518930626</v>
       </c>
       <c r="G55" t="n">
         <v>3</v>
@@ -3666,16 +3666,16 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1.910555351284071</v>
+        <v>1.913627989417931</v>
       </c>
       <c r="D57" t="n">
-        <v>0.006011968057233575</v>
+        <v>0.004722897818923137</v>
       </c>
       <c r="E57" t="n">
-        <v>1.903677557400715</v>
+        <v>1.908174481748671</v>
       </c>
       <c r="F57" t="n">
-        <v>1.914810166968486</v>
+        <v>1.916369039545121</v>
       </c>
       <c r="G57" t="n">
         <v>3</v>
@@ -3693,16 +3693,16 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>-1.182461181959481</v>
+        <v>-1.345187212637706</v>
       </c>
       <c r="D58" t="n">
-        <v>0.3183920969205906</v>
+        <v>0.250123308339837</v>
       </c>
       <c r="E58" t="n">
-        <v>-1.407794995259031</v>
+        <v>-1.490352437976927</v>
       </c>
       <c r="F58" t="n">
-        <v>-0.8182151986371745</v>
+        <v>-1.056371017032824</v>
       </c>
       <c r="G58" t="n">
         <v>3</v>
@@ -3720,16 +3720,16 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1232.239445833333</v>
+        <v>1242.106958333334</v>
       </c>
       <c r="D59" t="n">
-        <v>19.09283742742422</v>
+        <v>8.754022326823716</v>
       </c>
       <c r="E59" t="n">
-        <v>1210.25915</v>
+        <v>1231.9988</v>
       </c>
       <c r="F59" t="n">
-        <v>1244.7082375</v>
+        <v>1247.20296875</v>
       </c>
       <c r="G59" t="n">
         <v>3</v>
@@ -3774,16 +3774,16 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2217.333333333333</v>
+        <v>2231.333333333333</v>
       </c>
       <c r="D61" t="n">
-        <v>21.07921567168317</v>
+        <v>1.154700538379252</v>
       </c>
       <c r="E61" t="n">
-        <v>2193</v>
+        <v>2230</v>
       </c>
       <c r="F61" t="n">
-        <v>2230</v>
+        <v>2232</v>
       </c>
       <c r="G61" t="n">
         <v>3</v>
@@ -3855,13 +3855,13 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1.666666666666667</v>
+        <v>2</v>
       </c>
       <c r="D64" t="n">
-        <v>0.5773502691896257</v>
+        <v>0</v>
       </c>
       <c r="E64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F64" t="n">
         <v>2</v>
@@ -3882,16 +3882,16 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>0.07524951213338649</v>
+        <v>0.08963252272958623</v>
       </c>
       <c r="D65" t="n">
-        <v>0.02632622047753177</v>
+        <v>4.639811218715127e-05</v>
       </c>
       <c r="E65" t="n">
-        <v>0.04486316733961417</v>
+        <v>0.08960573476702509</v>
       </c>
       <c r="F65" t="n">
-        <v>0.09119927040583675</v>
+        <v>0.08968609865470852</v>
       </c>
       <c r="G65" t="n">
         <v>3</v>
@@ -3990,16 +3990,16 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>409.5439958333333</v>
+        <v>416.3356708333333</v>
       </c>
       <c r="D69" t="n">
-        <v>12.25192342615019</v>
+        <v>6.652912548264627</v>
       </c>
       <c r="E69" t="n">
-        <v>395.52620625</v>
+        <v>408.65355</v>
       </c>
       <c r="F69" t="n">
-        <v>418.20691875</v>
+        <v>420.17989375</v>
       </c>
       <c r="G69" t="n">
         <v>3</v>
@@ -4017,16 +4017,16 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2173.061849247566</v>
+        <v>2229.278683266341</v>
       </c>
       <c r="D70" t="n">
-        <v>89.04201667790794</v>
+        <v>23.95617066266183</v>
       </c>
       <c r="E70" t="n">
-        <v>2070.310236121836</v>
+        <v>2201.616662105195</v>
       </c>
       <c r="F70" t="n">
-        <v>2227.609443021797</v>
+        <v>2243.196594818203</v>
       </c>
       <c r="G70" t="n">
         <v>3</v>
@@ -4044,16 +4044,16 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>3221.880025694791</v>
+        <v>3300.1424951625</v>
       </c>
       <c r="D71" t="n">
-        <v>41.23548253186437</v>
+        <v>41.50135245593651</v>
       </c>
       <c r="E71" t="n">
-        <v>3174.495563967187</v>
+        <v>3252.221128535937</v>
       </c>
       <c r="F71" t="n">
-        <v>3249.62189971875</v>
+        <v>3324.241818851562</v>
       </c>
       <c r="G71" t="n">
         <v>3</v>
@@ -4071,16 +4071,16 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1048.818176447226</v>
+        <v>1070.863811896159</v>
       </c>
       <c r="D72" t="n">
-        <v>48.49010359926954</v>
+        <v>17.5451841250328</v>
       </c>
       <c r="E72" t="n">
-        <v>1013.913170376641</v>
+        <v>1050.604466430742</v>
       </c>
       <c r="F72" t="n">
-        <v>1104.185327845351</v>
+        <v>1081.045224033359</v>
       </c>
       <c r="G72" t="n">
         <v>3</v>
@@ -4098,16 +4098,16 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1048.818176447226</v>
+        <v>1070.863811896159</v>
       </c>
       <c r="D73" t="n">
-        <v>48.49010359926954</v>
+        <v>17.5451841250328</v>
       </c>
       <c r="E73" t="n">
-        <v>1013.913170376641</v>
+        <v>1050.604466430742</v>
       </c>
       <c r="F73" t="n">
-        <v>1104.185327845351</v>
+        <v>1081.045224033359</v>
       </c>
       <c r="G73" t="n">
         <v>3</v>
@@ -4125,16 +4125,16 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1912.61593123518</v>
+        <v>1962.857342472342</v>
       </c>
       <c r="D74" t="n">
-        <v>79.31994490510904</v>
+        <v>21.20212141275825</v>
       </c>
       <c r="E74" t="n">
-        <v>1821.083516713761</v>
+        <v>1938.375406145216</v>
       </c>
       <c r="F74" t="n">
-        <v>1961.213477164934</v>
+        <v>1975.176077320619</v>
       </c>
       <c r="G74" t="n">
         <v>3</v>
@@ -4152,16 +4152,16 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1480.717053841204</v>
+        <v>1516.86057718425</v>
       </c>
       <c r="D75" t="n">
-        <v>15.81310846844365</v>
+        <v>19.37365152828021</v>
       </c>
       <c r="E75" t="n">
-        <v>1462.634422279556</v>
+        <v>1494.489936287979</v>
       </c>
       <c r="F75" t="n">
-        <v>1491.953415473267</v>
+        <v>1528.110650676989</v>
       </c>
       <c r="G75" t="n">
         <v>3</v>
@@ -4206,16 +4206,16 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>122.3333333333333</v>
+        <v>121</v>
       </c>
       <c r="D77" t="n">
-        <v>2.309401076758503</v>
+        <v>0</v>
       </c>
       <c r="E77" t="n">
         <v>121</v>
       </c>
       <c r="F77" t="n">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="G77" t="n">
         <v>3</v>
@@ -4260,16 +4260,16 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>16.4426523297491</v>
+        <v>16.26344086021505</v>
       </c>
       <c r="D79" t="n">
-        <v>0.3104033705320576</v>
+        <v>0</v>
       </c>
       <c r="E79" t="n">
         <v>16.26344086021505</v>
       </c>
       <c r="F79" t="n">
-        <v>16.8010752688172</v>
+        <v>16.26344086021505</v>
       </c>
       <c r="G79" t="n">
         <v>3</v>
@@ -4287,13 +4287,13 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>28.58422939068101</v>
+        <v>28.76344086021506</v>
       </c>
       <c r="D80" t="n">
-        <v>0.3104033705320556</v>
+        <v>0</v>
       </c>
       <c r="E80" t="n">
-        <v>28.22580645161291</v>
+        <v>28.76344086021506</v>
       </c>
       <c r="F80" t="n">
         <v>28.76344086021506</v>
@@ -4314,16 +4314,16 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>188.5771333333333</v>
+        <v>186.812075</v>
       </c>
       <c r="D81" t="n">
-        <v>2.528581770667209</v>
+        <v>0.04513352585661034</v>
       </c>
       <c r="E81" t="n">
-        <v>186.9453875</v>
+        <v>186.768075</v>
       </c>
       <c r="F81" t="n">
-        <v>191.48985625</v>
+        <v>186.8582625</v>
       </c>
       <c r="G81" t="n">
         <v>3</v>
@@ -4341,16 +4341,16 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>6.630112499999999</v>
+        <v>6.602374999999999</v>
       </c>
       <c r="D82" t="n">
-        <v>0.0480427592749413</v>
+        <v>0</v>
       </c>
       <c r="E82" t="n">
         <v>6.602374999999999</v>
       </c>
       <c r="F82" t="n">
-        <v>6.685587499999999</v>
+        <v>6.602374999999999</v>
       </c>
       <c r="G82" t="n">
         <v>3</v>
@@ -4368,16 +4368,16 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1.091140742607527</v>
+        <v>1.099658747759857</v>
       </c>
       <c r="D83" t="n">
-        <v>0.01896453145771046</v>
+        <v>0.01177129531145826</v>
       </c>
       <c r="E83" t="n">
-        <v>1.069427234543011</v>
+        <v>1.086066633064516</v>
       </c>
       <c r="F83" t="n">
-        <v>1.104456384408602</v>
+        <v>1.106519665658602</v>
       </c>
       <c r="G83" t="n">
         <v>3</v>
@@ -4422,16 +4422,16 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>609.0078666666666</v>
+        <v>610.7729250000001</v>
       </c>
       <c r="D85" t="n">
-        <v>2.528581770667142</v>
+        <v>0.0451335258565958</v>
       </c>
       <c r="E85" t="n">
-        <v>606.09514375</v>
+        <v>610.7267375</v>
       </c>
       <c r="F85" t="n">
-        <v>610.6396124999999</v>
+        <v>610.816925</v>
       </c>
       <c r="G85" t="n">
         <v>3</v>
@@ -4449,16 +4449,16 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>623.2315791666666</v>
+        <v>631.3340333333333</v>
       </c>
       <c r="D86" t="n">
-        <v>16.59563381548259</v>
+        <v>8.75581690384211</v>
       </c>
       <c r="E86" t="n">
-        <v>604.1640062500001</v>
+        <v>621.2236875</v>
       </c>
       <c r="F86" t="n">
-        <v>634.4193937499999</v>
+        <v>636.3923687500001</v>
       </c>
       <c r="G86" t="n">
         <v>3</v>
@@ -4476,16 +4476,16 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>188.5771333333333</v>
+        <v>186.812075</v>
       </c>
       <c r="D87" t="n">
-        <v>2.528581770667209</v>
+        <v>0.04513352585661034</v>
       </c>
       <c r="E87" t="n">
-        <v>186.9453875</v>
+        <v>186.768075</v>
       </c>
       <c r="F87" t="n">
-        <v>191.48985625</v>
+        <v>186.8582625</v>
       </c>
       <c r="G87" t="n">
         <v>3</v>
@@ -4503,16 +4503,16 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>49.42871587296251</v>
+        <v>49.17396501204887</v>
       </c>
       <c r="D88" t="n">
-        <v>0.5684828700705817</v>
+        <v>0.3481350205221764</v>
       </c>
       <c r="E88" t="n">
-        <v>49.03067444751284</v>
+        <v>48.97100320565312</v>
       </c>
       <c r="F88" t="n">
-        <v>50.0797819830571</v>
+        <v>49.57595027689963</v>
       </c>
       <c r="G88" t="n">
         <v>3</v>
@@ -4530,16 +4530,16 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>66.76922892384259</v>
+        <v>66.48290839294668</v>
       </c>
       <c r="D89" t="n">
-        <v>0.4850512999744201</v>
+        <v>0.300625115787693</v>
       </c>
       <c r="E89" t="n">
-        <v>66.40120904237206</v>
+        <v>66.3079579452959</v>
       </c>
       <c r="F89" t="n">
-        <v>67.31888321191374</v>
+        <v>66.83003668510067</v>
       </c>
       <c r="G89" t="n">
         <v>3</v>
@@ -4557,16 +4557,16 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>3.567837628096528</v>
+        <v>3.649930514995936</v>
       </c>
       <c r="D90" t="n">
-        <v>0.131801442555127</v>
+        <v>0.03923392199351299</v>
       </c>
       <c r="E90" t="n">
-        <v>3.415817231783976</v>
+        <v>3.6046273285328</v>
       </c>
       <c r="F90" t="n">
-        <v>3.65009038889513</v>
+        <v>3.672710977183351</v>
       </c>
       <c r="G90" t="n">
         <v>3</v>
@@ -4611,16 +4611,16 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>13.6301125</v>
+        <v>13.602375</v>
       </c>
       <c r="D92" t="n">
-        <v>0.04804275927494181</v>
+        <v>0</v>
       </c>
       <c r="E92" t="n">
         <v>13.602375</v>
       </c>
       <c r="F92" t="n">
-        <v>13.6855875</v>
+        <v>13.602375</v>
       </c>
       <c r="G92" t="n">
         <v>3</v>
@@ -4638,13 +4638,13 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>9.816475064097272</v>
+        <v>10.00000000000001</v>
       </c>
       <c r="D93" t="n">
-        <v>0.317874513439365</v>
+        <v>0</v>
       </c>
       <c r="E93" t="n">
-        <v>9.449425192291795</v>
+        <v>10.00000000000001</v>
       </c>
       <c r="F93" t="n">
         <v>10.00000000000001</v>
@@ -4746,16 +4746,16 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>3.676771736111112</v>
+        <v>3.662524305555556</v>
       </c>
       <c r="D97" t="n">
-        <v>0.008238829965382636</v>
+        <v>0.002459369002651483</v>
       </c>
       <c r="E97" t="n">
-        <v>3.667258750000001</v>
+        <v>3.660469166666667</v>
       </c>
       <c r="F97" t="n">
-        <v>3.681603333333334</v>
+        <v>3.665249166666667</v>
       </c>
       <c r="G97" t="n">
         <v>3</v>
@@ -4773,16 +4773,16 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>27.73510261529648</v>
+        <v>28.01512791493118</v>
       </c>
       <c r="D98" t="n">
-        <v>0.1619296069350606</v>
+        <v>0.04833752578715014</v>
       </c>
       <c r="E98" t="n">
-        <v>27.64014026720212</v>
+        <v>27.96157228985714</v>
       </c>
       <c r="F98" t="n">
-        <v>27.92207505048732</v>
+        <v>28.05552052333226</v>
       </c>
       <c r="G98" t="n">
         <v>3</v>
@@ -4827,16 +4827,16 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>1.268379623842593</v>
+        <v>1.252904479166667</v>
       </c>
       <c r="D100" t="n">
-        <v>0.002275911157233519</v>
+        <v>0.004214815184314371</v>
       </c>
       <c r="E100" t="n">
-        <v>1.266953602430556</v>
+        <v>1.250416657986111</v>
       </c>
       <c r="F100" t="n">
-        <v>1.271004340277778</v>
+        <v>1.257770920138889</v>
       </c>
       <c r="G100" t="n">
         <v>3</v>
@@ -4854,16 +4854,16 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>26.21624595895449</v>
+        <v>27.1164608844032</v>
       </c>
       <c r="D101" t="n">
-        <v>0.1323935404574366</v>
+        <v>0.2451828151778211</v>
       </c>
       <c r="E101" t="n">
-        <v>26.06356183486355</v>
+        <v>26.8333719124581</v>
       </c>
       <c r="F101" t="n">
-        <v>26.29919999822252</v>
+        <v>27.26118158365893</v>
       </c>
       <c r="G101" t="n">
         <v>3</v>
@@ -4908,16 +4908,16 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>2.940716946404779</v>
+        <v>2.977939224066652</v>
       </c>
       <c r="D103" t="n">
-        <v>0.0103505951393558</v>
+        <v>0.007537462055057653</v>
       </c>
       <c r="E103" t="n">
-        <v>2.930153742566731</v>
+        <v>2.969249648454104</v>
       </c>
       <c r="F103" t="n">
-        <v>2.950840950955322</v>
+        <v>2.982710381415455</v>
       </c>
       <c r="G103" t="n">
         <v>3</v>
@@ -4935,16 +4935,16 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>2.671845496345397</v>
+        <v>1.439909319801211</v>
       </c>
       <c r="D104" t="n">
-        <v>0.3425709924784209</v>
+        <v>0.2494654483346253</v>
       </c>
       <c r="E104" t="n">
-        <v>2.336773914466162</v>
+        <v>1.281999548793387</v>
       </c>
       <c r="F104" t="n">
-        <v>3.021453144391929</v>
+        <v>1.727505975039728</v>
       </c>
       <c r="G104" t="n">
         <v>3</v>
@@ -4962,16 +4962,16 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>324.4826708333333</v>
+        <v>335.624775</v>
       </c>
       <c r="D105" t="n">
-        <v>1.638656033208081</v>
+        <v>3.034666932706274</v>
       </c>
       <c r="E105" t="n">
-        <v>322.592875</v>
+        <v>332.1209375</v>
       </c>
       <c r="F105" t="n">
-        <v>325.50940625</v>
+        <v>337.41600625</v>
       </c>
       <c r="G105" t="n">
         <v>3</v>
@@ -5016,16 +5016,16 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>2082</v>
+        <v>2159.666666666667</v>
       </c>
       <c r="D107" t="n">
-        <v>39.05124837953327</v>
+        <v>0.5773502691896258</v>
       </c>
       <c r="E107" t="n">
-        <v>2057</v>
+        <v>2159</v>
       </c>
       <c r="F107" t="n">
-        <v>2127</v>
+        <v>2160</v>
       </c>
       <c r="G107" t="n">
         <v>3</v>
@@ -5097,16 +5097,16 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>309.6666666666667</v>
+        <v>337</v>
       </c>
       <c r="D110" t="n">
-        <v>21.93931022920578</v>
+        <v>0</v>
       </c>
       <c r="E110" t="n">
-        <v>285</v>
+        <v>337</v>
       </c>
       <c r="F110" t="n">
-        <v>327</v>
+        <v>337</v>
       </c>
       <c r="G110" t="n">
         <v>3</v>
@@ -5124,16 +5124,16 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>14.86869692542814</v>
+        <v>15.60426066022793</v>
       </c>
       <c r="D111" t="n">
-        <v>0.9070599501497216</v>
+        <v>0.004172178493068751</v>
       </c>
       <c r="E111" t="n">
-        <v>13.82153249272551</v>
+        <v>15.60185185185185</v>
       </c>
       <c r="F111" t="n">
-        <v>15.41079241614001</v>
+        <v>15.60907827698009</v>
       </c>
       <c r="G111" t="n">
         <v>3</v>
@@ -5232,16 +5232,16 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>313.4007458333334</v>
+        <v>324.54285</v>
       </c>
       <c r="D115" t="n">
-        <v>1.638656033208114</v>
+        <v>3.034666932706274</v>
       </c>
       <c r="E115" t="n">
-        <v>311.51095</v>
+        <v>321.0390125</v>
       </c>
       <c r="F115" t="n">
-        <v>314.42748125</v>
+        <v>326.33408125</v>
       </c>
       <c r="G115" t="n">
         <v>3</v>
@@ -5259,16 +5259,16 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>460.2750429537957</v>
+        <v>496.7206654588046</v>
       </c>
       <c r="D116" t="n">
-        <v>1.455149434887337</v>
+        <v>6.841099493582388</v>
       </c>
       <c r="E116" t="n">
-        <v>458.6090682438653</v>
+        <v>488.8222426560772</v>
       </c>
       <c r="F116" t="n">
-        <v>461.2973873188162</v>
+        <v>500.7786435973168</v>
       </c>
       <c r="G116" t="n">
         <v>3</v>
@@ -5286,16 +5286,16 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>974.222499582398</v>
+        <v>1020.98021735608</v>
       </c>
       <c r="D117" t="n">
-        <v>5.459133964477632</v>
+        <v>12.20621537577031</v>
       </c>
       <c r="E117" t="n">
-        <v>967.9858473513925</v>
+        <v>1006.887396834205</v>
       </c>
       <c r="F117" t="n">
-        <v>978.1347213801125</v>
+        <v>1028.216367184205</v>
       </c>
       <c r="G117" t="n">
         <v>3</v>
@@ -5313,16 +5313,16 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>513.9474566286023</v>
+        <v>524.2595518972754</v>
       </c>
       <c r="D118" t="n">
-        <v>4.004221117443201</v>
+        <v>5.365116860464414</v>
       </c>
       <c r="E118" t="n">
-        <v>509.3767791075272</v>
+        <v>518.0651541781278</v>
       </c>
       <c r="F118" t="n">
-        <v>516.8373340612964</v>
+        <v>527.4377235868881</v>
       </c>
       <c r="G118" t="n">
         <v>3</v>
@@ -5340,16 +5340,16 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>513.9474566286021</v>
+        <v>524.2595518972753</v>
       </c>
       <c r="D119" t="n">
-        <v>4.004221117443177</v>
+        <v>5.36511686046435</v>
       </c>
       <c r="E119" t="n">
-        <v>509.3767791075272</v>
+        <v>518.0651541781278</v>
       </c>
       <c r="F119" t="n">
-        <v>516.8373340612964</v>
+        <v>527.4377235868881</v>
       </c>
       <c r="G119" t="n">
         <v>3</v>
@@ -5367,16 +5367,16 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>406.3711715386876</v>
+        <v>438.9634495105784</v>
       </c>
       <c r="D120" t="n">
-        <v>1.348345504242473</v>
+        <v>6.084979711751679</v>
       </c>
       <c r="E120" t="n">
-        <v>404.8383385241723</v>
+        <v>431.9380191112659</v>
       </c>
       <c r="F120" t="n">
-        <v>407.3739200391661</v>
+        <v>442.5734985211225</v>
       </c>
       <c r="G120" t="n">
         <v>3</v>
@@ -5394,16 +5394,16 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>460.1593140836449</v>
+        <v>481.6115007039268</v>
       </c>
       <c r="D121" t="n">
-        <v>2.676130327517698</v>
+        <v>5.725047704373653</v>
       </c>
       <c r="E121" t="n">
-        <v>457.1075588158497</v>
+        <v>475.0015866446969</v>
       </c>
       <c r="F121" t="n">
-        <v>462.1056270502312</v>
+        <v>485.0056110540053</v>
       </c>
       <c r="G121" t="n">
         <v>3</v>
@@ -5610,16 +5610,16 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>0.4399316261574073</v>
+        <v>0.4554067708333333</v>
       </c>
       <c r="D129" t="n">
-        <v>0.002275911157233448</v>
+        <v>0.00421481518431429</v>
       </c>
       <c r="E129" t="n">
-        <v>0.4373069097222222</v>
+        <v>0.4505403298611111</v>
       </c>
       <c r="F129" t="n">
-        <v>0.4413576475694444</v>
+        <v>0.4578945920138889</v>
       </c>
       <c r="G129" t="n">
         <v>3</v>
@@ -5691,16 +5691,16 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>316.1468458333333</v>
+        <v>327.28895</v>
       </c>
       <c r="D132" t="n">
-        <v>1.638656033208081</v>
+        <v>3.034666932706274</v>
       </c>
       <c r="E132" t="n">
-        <v>314.25705</v>
+        <v>323.7851125</v>
       </c>
       <c r="F132" t="n">
-        <v>317.17358125</v>
+        <v>329.08018125</v>
       </c>
       <c r="G132" t="n">
         <v>3</v>
@@ -5745,16 +5745,16 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>2.569002257328714</v>
+        <v>2.483810004007269</v>
       </c>
       <c r="D134" t="n">
-        <v>0.01301112246979353</v>
+        <v>0.02257598920973822</v>
       </c>
       <c r="E134" t="n">
-        <v>2.560855336265724</v>
+        <v>2.470488905562997</v>
       </c>
       <c r="F134" t="n">
-        <v>2.584007783804897</v>
+        <v>2.509876391036022</v>
       </c>
       <c r="G134" t="n">
         <v>3</v>
@@ -5772,16 +5772,16 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>3.415317660885096</v>
+        <v>3.302060225431587</v>
       </c>
       <c r="D135" t="n">
-        <v>0.01729742207592626</v>
+        <v>0.03001327633714944</v>
       </c>
       <c r="E135" t="n">
-        <v>3.404486871107124</v>
+        <v>3.284350710911184</v>
       </c>
       <c r="F135" t="n">
-        <v>3.435266510458422</v>
+        <v>3.33671375355551</v>
       </c>
       <c r="G135" t="n">
         <v>3</v>
@@ -5799,16 +5799,16 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>55.21649542232421</v>
+        <v>59.58866284486595</v>
       </c>
       <c r="D136" t="n">
-        <v>0.1745657370311018</v>
+        <v>0.8206865539502656</v>
       </c>
       <c r="E136" t="n">
-        <v>55.01663821443772</v>
+        <v>58.64113541923891</v>
       </c>
       <c r="F136" t="n">
-        <v>55.3391400753754</v>
+        <v>60.07547466475326</v>
       </c>
       <c r="G136" t="n">
         <v>3</v>
@@ -5915,8 +5915,8 @@
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
     <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="38" customWidth="1" min="9" max="9"/>
     <col width="45" customWidth="1" min="10" max="10"/>
@@ -5995,22 +5995,22 @@
         <v>100</v>
       </c>
       <c r="D2" t="n">
-        <v>98.34229390681004</v>
+        <v>99.91039426523297</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>69.75806451612904</v>
       </c>
       <c r="F2" t="n">
-        <v>0.06712516056355411</v>
+        <v>-0.01425699403397513</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1012544802867383</v>
+        <v>0.02654569892473118</v>
       </c>
       <c r="H2" t="n">
-        <v>0.7729736917261344</v>
+        <v>0.9177981735906263</v>
       </c>
       <c r="I2" t="n">
-        <v>0.1114596427531362</v>
+        <v>0.02735624622983871</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -6034,22 +6034,22 @@
         <v>100</v>
       </c>
       <c r="D3" t="n">
-        <v>98.34229390681004</v>
+        <v>100</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>69.89247311827957</v>
       </c>
       <c r="F3" t="n">
-        <v>0.07668599817708474</v>
+        <v>-0.007123705465796419</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1052867383512545</v>
+        <v>0.02553763440860215</v>
       </c>
       <c r="H3" t="n">
-        <v>0.7639478453060661</v>
+        <v>0.9175699017494118</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1189575117853943</v>
+        <v>0.02725761551747313</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -6073,22 +6073,22 @@
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>99.64157706093189</v>
+        <v>99.91039426523297</v>
       </c>
       <c r="E4" t="n">
-        <v>86.15591397849462</v>
+        <v>99.59677419354838</v>
       </c>
       <c r="F4" t="n">
-        <v>0.2773263420148495</v>
+        <v>-0.0008970619638014954</v>
       </c>
       <c r="G4" t="n">
-        <v>0.02956989247311828</v>
+        <v>0.001232078853046595</v>
       </c>
       <c r="H4" t="n">
-        <v>0.9449686425610018</v>
+        <v>0.9997054860548853</v>
       </c>
       <c r="I4" t="n">
-        <v>0.03221253637096774</v>
+        <v>0.0003722642249103943</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -6112,22 +6112,22 @@
         <v>100</v>
       </c>
       <c r="D5" t="n">
-        <v>98.11827956989248</v>
+        <v>99.91039426523297</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>69.75806451612904</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0715212180488297</v>
+        <v>-0.01415153593572612</v>
       </c>
       <c r="G5" t="n">
-        <v>0.102486559139785</v>
+        <v>0.02632168458781362</v>
       </c>
       <c r="H5" t="n">
-        <v>0.5590336560960016</v>
+        <v>0.83100643885571</v>
       </c>
       <c r="I5" t="n">
-        <v>0.1400403701836918</v>
+        <v>0.03385866095430108</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -6151,22 +6151,22 @@
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>98.16308243727599</v>
+        <v>100</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>69.89247311827957</v>
       </c>
       <c r="F6" t="n">
-        <v>0.08375485925883552</v>
+        <v>-0.01000216275479539</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1047267025089606</v>
+        <v>0.02542562724014337</v>
       </c>
       <c r="H6" t="n">
-        <v>0.5608070941536235</v>
+        <v>0.8364075428625766</v>
       </c>
       <c r="I6" t="n">
-        <v>0.1421606574820788</v>
+        <v>0.03210409106182796</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -6190,22 +6190,22 @@
         <v>100</v>
       </c>
       <c r="D7" t="n">
-        <v>99.77598566308244</v>
+        <v>99.91039426523297</v>
       </c>
       <c r="E7" t="n">
-        <v>87.23118279569893</v>
+        <v>99.46236559139786</v>
       </c>
       <c r="F7" t="n">
-        <v>0.3067753591573523</v>
+        <v>-0.001268921611417179</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0246415770609319</v>
+        <v>0.001344086021505376</v>
       </c>
       <c r="H7" t="n">
-        <v>0.9078409983768124</v>
+        <v>0.993519303223515</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0326178959453405</v>
+        <v>0.002303444220430108</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -6229,22 +6229,22 @@
         <v>100</v>
       </c>
       <c r="D8" t="n">
-        <v>91.99074074074073</v>
+        <v>99.9537037037037</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>79.02777777777777</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1451919906352565</v>
+        <v>-0.01441783031007261</v>
       </c>
       <c r="G8" t="n">
-        <v>0.209837962962963</v>
+        <v>0.01886574074074074</v>
       </c>
       <c r="H8" t="n">
-        <v>0.8322646277353848</v>
+        <v>0.9877564099259014</v>
       </c>
       <c r="I8" t="n">
-        <v>0.2207584246689815</v>
+        <v>0.02008501925231481</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -6268,22 +6268,22 @@
         <v>100</v>
       </c>
       <c r="D9" t="n">
-        <v>94.72222222222221</v>
+        <v>100</v>
       </c>
       <c r="E9" t="n">
-        <v>0.5555555555555556</v>
+        <v>79.30555555555556</v>
       </c>
       <c r="F9" t="n">
-        <v>0.194146265349361</v>
+        <v>-0.008316427999044647</v>
       </c>
       <c r="G9" t="n">
-        <v>0.2018518518518519</v>
+        <v>0.01793981481481481</v>
       </c>
       <c r="H9" t="n">
-        <v>0.8508681533098651</v>
+        <v>0.9898557664284198</v>
       </c>
       <c r="I9" t="n">
-        <v>0.2187748829467593</v>
+        <v>0.0186503751550926</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -6307,22 +6307,22 @@
         <v>100</v>
       </c>
       <c r="D10" t="n">
-        <v>94.21296296296296</v>
+        <v>99.9537037037037</v>
       </c>
       <c r="E10" t="n">
-        <v>33.33333333333333</v>
+        <v>99.58333333333333</v>
       </c>
       <c r="F10" t="n">
-        <v>0.3133066026186074</v>
+        <v>0.2877375374069236</v>
       </c>
       <c r="G10" t="n">
-        <v>0.1885416666666667</v>
+        <v>0.00162037037037037</v>
       </c>
       <c r="H10" t="n">
-        <v>0.8539365111688423</v>
+        <v>0.997913885286305</v>
       </c>
       <c r="I10" t="n">
-        <v>0.1944794055740741</v>
+        <v>0.001744053819444445</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>

</xml_diff>